<commit_message>
Update demo data and install script
</commit_message>
<xml_diff>
--- a/data/seed/demo_compleet.xlsx
+++ b/data/seed/demo_compleet.xlsx
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,8 +89,13 @@
       <color rgb="001E3A5F"/>
       <sz val="14"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00CBD5E1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -157,6 +162,11 @@
         <fgColor rgb="00BFDBFE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -170,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -279,6 +289,12 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="10" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -666,17 +682,13 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TABS IN DIT BESTAND</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -798,17 +810,13 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-      <c r="B15" t="inlineStr"/>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>EINDSCORE LEVERANCIER ALPHA</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -858,17 +866,13 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
-    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>IMPORT-INSTRUCTIE</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1132,12 +1136,16 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Requirements scoring (gewicht: 75%)</t>
         </is>
       </c>
+      <c r="B4" t="n">
+        <v>3.577</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1161,7 +1169,7 @@
         </is>
       </c>
       <c r="B6" s="40" t="n">
-        <v>3.617</v>
+        <v>3.5</v>
       </c>
       <c r="C6" s="41" t="inlineStr">
         <is>
@@ -1176,7 +1184,7 @@
         </is>
       </c>
       <c r="B7" s="40" t="n">
-        <v>3.314</v>
+        <v>3.309</v>
       </c>
       <c r="C7" s="41" t="inlineStr">
         <is>
@@ -1191,7 +1199,7 @@
         </is>
       </c>
       <c r="B8" s="40" t="n">
-        <v>3.72</v>
+        <v>3.667</v>
       </c>
       <c r="C8" s="41" t="inlineStr">
         <is>
@@ -1206,7 +1214,7 @@
         </is>
       </c>
       <c r="B9" s="40" t="n">
-        <v>3.927</v>
+        <v>3.909</v>
       </c>
       <c r="C9" s="41" t="inlineStr">
         <is>
@@ -1221,7 +1229,7 @@
         </is>
       </c>
       <c r="B10" s="40" t="n">
-        <v>3.3</v>
+        <v>3.278</v>
       </c>
       <c r="C10" s="41" t="inlineStr">
         <is>
@@ -1236,9 +1244,10 @@
         </is>
       </c>
       <c r="B11" s="42" t="n">
-        <v>3.539</v>
-      </c>
-    </row>
+        <v>3.503</v>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -7639,7 +7648,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7647,6 +7656,7 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7675,6 +7685,11 @@
           <t>Opmerking</t>
         </is>
       </c>
+      <c r="F1" s="45" t="inlineStr">
+        <is>
+          <t>Scopes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="16" t="inlineStr">
@@ -7702,6 +7717,11 @@
           <t>Kritische denker, focus op NFR en licentiekosten</t>
         </is>
       </c>
+      <c r="F2" s="16" t="inlineStr">
+        <is>
+          <t>FUNC;NFR;VEND;IMPL;SUP;LIC</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
@@ -7729,6 +7749,11 @@
           <t>Finance &amp; inkoop key-user, positief over de demo</t>
         </is>
       </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>FUNC;NFR;LIC</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
@@ -7756,6 +7781,11 @@
           <t>Projectleider ERP-traject, let op implementatieaanpak</t>
         </is>
       </c>
+      <c r="F4" s="16" t="inlineStr">
+        <is>
+          <t>FUNC;VEND;IMPL</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
@@ -7783,6 +7813,11 @@
           <t>Productie key-user, focus op MRP en shop floor</t>
         </is>
       </c>
+      <c r="F5" s="17" t="inlineStr">
+        <is>
+          <t>FUNC;IMPL;SUP</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
@@ -7808,6 +7843,11 @@
       <c r="E6" s="16" t="inlineStr">
         <is>
           <t>Logistiek key-user, geïnteresseerd in WMS-integratie</t>
+        </is>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>FUNC;VEND;LIC</t>
         </is>
       </c>
     </row>
@@ -9154,15 +9194,9 @@
       <c r="H24" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I24" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J24" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="K24" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I24" s="46" t="n"/>
+      <c r="J24" s="46" t="n"/>
+      <c r="K24" s="46" t="n"/>
       <c r="L24" s="22" t="n">
         <v>4</v>
       </c>
@@ -9209,17 +9243,11 @@
       <c r="H25" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I25" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J25" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="K25" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I25" s="46" t="n"/>
+      <c r="J25" s="46" t="n"/>
+      <c r="K25" s="46" t="n"/>
       <c r="L25" s="25" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="M25" s="21" t="inlineStr">
         <is>
@@ -9264,17 +9292,11 @@
       <c r="H26" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I26" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J26" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="K26" s="21" t="n">
-        <v>5</v>
-      </c>
+      <c r="I26" s="46" t="n"/>
+      <c r="J26" s="46" t="n"/>
+      <c r="K26" s="46" t="n"/>
       <c r="L26" s="22" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="M26" s="23" t="inlineStr">
         <is>
@@ -9319,17 +9341,11 @@
       <c r="H27" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="I27" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J27" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="K27" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I27" s="46" t="n"/>
+      <c r="J27" s="46" t="n"/>
+      <c r="K27" s="46" t="n"/>
       <c r="L27" s="25" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="M27" s="21" t="inlineStr">
         <is>
@@ -9374,17 +9390,11 @@
       <c r="H28" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="I28" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="J28" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="K28" s="21" t="n">
-        <v>2</v>
-      </c>
+      <c r="I28" s="46" t="n"/>
+      <c r="J28" s="46" t="n"/>
+      <c r="K28" s="46" t="n"/>
       <c r="L28" s="27" t="n">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="M28" s="23" t="inlineStr">
         <is>
@@ -9429,15 +9439,9 @@
       <c r="H29" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I29" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J29" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="K29" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I29" s="46" t="n"/>
+      <c r="J29" s="46" t="n"/>
+      <c r="K29" s="46" t="n"/>
       <c r="L29" s="22" t="n">
         <v>4</v>
       </c>
@@ -9484,17 +9488,11 @@
       <c r="H30" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="I30" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="J30" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="K30" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I30" s="46" t="n"/>
+      <c r="J30" s="46" t="n"/>
+      <c r="K30" s="46" t="n"/>
       <c r="L30" s="25" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M30" s="23" t="inlineStr">
         <is>
@@ -9539,15 +9537,9 @@
       <c r="H31" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="I31" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="J31" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="K31" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I31" s="46" t="n"/>
+      <c r="J31" s="46" t="n"/>
+      <c r="K31" s="46" t="n"/>
       <c r="L31" s="25" t="n">
         <v>3</v>
       </c>
@@ -9594,17 +9586,11 @@
       <c r="H32" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="I32" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J32" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="K32" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I32" s="46" t="n"/>
+      <c r="J32" s="46" t="n"/>
+      <c r="K32" s="46" t="n"/>
       <c r="L32" s="22" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="M32" s="23" t="inlineStr">
         <is>
@@ -9649,17 +9635,11 @@
       <c r="H33" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="I33" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="J33" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="K33" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I33" s="46" t="n"/>
+      <c r="J33" s="46" t="n"/>
+      <c r="K33" s="46" t="n"/>
       <c r="L33" s="25" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M33" s="21" t="inlineStr">
         <is>
@@ -9704,17 +9684,11 @@
       <c r="H34" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I34" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J34" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="K34" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I34" s="46" t="n"/>
+      <c r="J34" s="46" t="n"/>
+      <c r="K34" s="46" t="n"/>
       <c r="L34" s="25" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="M34" s="23" t="inlineStr">
         <is>
@@ -9759,17 +9733,11 @@
       <c r="H35" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I35" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J35" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="K35" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I35" s="46" t="n"/>
+      <c r="J35" s="46" t="n"/>
+      <c r="K35" s="46" t="n"/>
       <c r="L35" s="22" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="M35" s="21" t="inlineStr">
         <is>
@@ -9811,20 +9779,16 @@
       <c r="G36" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H36" s="21" t="n">
-        <v>5</v>
-      </c>
+      <c r="H36" s="46" t="n"/>
       <c r="I36" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="J36" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="J36" s="46" t="n"/>
       <c r="K36" s="21" t="n">
         <v>4</v>
       </c>
       <c r="L36" s="22" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="M36" s="23" t="inlineStr">
         <is>
@@ -9866,20 +9830,16 @@
       <c r="G37" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H37" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H37" s="46" t="n"/>
       <c r="I37" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="J37" s="21" t="n">
-        <v>5</v>
-      </c>
+      <c r="J37" s="46" t="n"/>
       <c r="K37" s="21" t="n">
         <v>4</v>
       </c>
       <c r="L37" s="22" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="M37" s="21" t="inlineStr">
         <is>
@@ -9921,15 +9881,11 @@
       <c r="G38" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H38" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H38" s="46" t="n"/>
       <c r="I38" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="J38" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="J38" s="46" t="n"/>
       <c r="K38" s="21" t="n">
         <v>4</v>
       </c>
@@ -9976,15 +9932,11 @@
       <c r="G39" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H39" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="H39" s="46" t="n"/>
       <c r="I39" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="J39" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="J39" s="46" t="n"/>
       <c r="K39" s="21" t="n">
         <v>3</v>
       </c>
@@ -10031,20 +9983,16 @@
       <c r="G40" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H40" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H40" s="46" t="n"/>
       <c r="I40" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="J40" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="J40" s="46" t="n"/>
       <c r="K40" s="21" t="n">
         <v>4</v>
       </c>
       <c r="L40" s="25" t="n">
-        <v>3.8</v>
+        <v>3.67</v>
       </c>
       <c r="M40" s="23" t="inlineStr">
         <is>
@@ -10086,20 +10034,16 @@
       <c r="G41" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="H41" s="21" t="n">
-        <v>2</v>
-      </c>
+      <c r="H41" s="46" t="n"/>
       <c r="I41" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="J41" s="21" t="n">
-        <v>1</v>
-      </c>
+      <c r="J41" s="46" t="n"/>
       <c r="K41" s="21" t="n">
         <v>2</v>
       </c>
       <c r="L41" s="29" t="n">
-        <v>1.4</v>
+        <v>1.33</v>
       </c>
       <c r="M41" s="21" t="inlineStr">
         <is>
@@ -10141,20 +10085,16 @@
       <c r="G42" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="H42" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H42" s="46" t="n"/>
       <c r="I42" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="J42" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="J42" s="46" t="n"/>
       <c r="K42" s="21" t="n">
         <v>4</v>
       </c>
       <c r="L42" s="22" t="n">
-        <v>4.2</v>
+        <v>4.33</v>
       </c>
       <c r="M42" s="23" t="inlineStr">
         <is>
@@ -10196,20 +10136,16 @@
       <c r="G43" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="H43" s="21" t="n">
-        <v>1</v>
-      </c>
+      <c r="H43" s="46" t="n"/>
       <c r="I43" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="J43" s="21" t="n">
-        <v>1</v>
-      </c>
+      <c r="J43" s="46" t="n"/>
       <c r="K43" s="21" t="n">
         <v>1</v>
       </c>
       <c r="L43" s="29" t="n">
-        <v>1.4</v>
+        <v>1.67</v>
       </c>
       <c r="M43" s="21" t="inlineStr">
         <is>
@@ -10251,15 +10187,11 @@
       <c r="G44" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="H44" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="H44" s="46" t="n"/>
       <c r="I44" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="J44" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="J44" s="46" t="n"/>
       <c r="K44" s="21" t="n">
         <v>4</v>
       </c>
@@ -10306,20 +10238,16 @@
       <c r="G45" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H45" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H45" s="46" t="n"/>
       <c r="I45" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="J45" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="J45" s="46" t="n"/>
       <c r="K45" s="21" t="n">
         <v>5</v>
       </c>
       <c r="L45" s="22" t="n">
-        <v>4.2</v>
+        <v>4.33</v>
       </c>
       <c r="M45" s="21" t="inlineStr">
         <is>
@@ -10361,20 +10289,16 @@
       <c r="G46" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H46" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="H46" s="46" t="n"/>
       <c r="I46" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="J46" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="J46" s="46" t="n"/>
       <c r="K46" s="21" t="n">
         <v>4</v>
       </c>
       <c r="L46" s="25" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="M46" s="23" t="inlineStr">
         <is>
@@ -10416,20 +10340,16 @@
       <c r="G47" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="H47" s="21" t="n">
-        <v>2</v>
-      </c>
+      <c r="H47" s="46" t="n"/>
       <c r="I47" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="J47" s="21" t="n">
-        <v>1</v>
-      </c>
+      <c r="J47" s="46" t="n"/>
       <c r="K47" s="21" t="n">
         <v>1</v>
       </c>
       <c r="L47" s="29" t="n">
-        <v>1.4</v>
+        <v>1.33</v>
       </c>
       <c r="M47" s="21" t="inlineStr">
         <is>
@@ -10471,15 +10391,11 @@
       <c r="G48" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H48" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H48" s="46" t="n"/>
       <c r="I48" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="J48" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="J48" s="46" t="n"/>
       <c r="K48" s="21" t="n">
         <v>4</v>
       </c>
@@ -10526,20 +10442,16 @@
       <c r="G49" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H49" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H49" s="46" t="n"/>
       <c r="I49" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="J49" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="J49" s="46" t="n"/>
       <c r="K49" s="21" t="n">
         <v>4</v>
       </c>
       <c r="L49" s="25" t="n">
-        <v>3.8</v>
+        <v>3.67</v>
       </c>
       <c r="M49" s="21" t="inlineStr">
         <is>
@@ -10581,18 +10493,14 @@
       <c r="G50" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H50" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H50" s="46" t="n"/>
       <c r="I50" s="21" t="n">
         <v>4</v>
       </c>
       <c r="J50" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K50" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K50" s="46" t="n"/>
       <c r="L50" s="22" t="n">
         <v>4</v>
       </c>
@@ -10636,20 +10544,16 @@
       <c r="G51" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H51" s="21" t="n">
-        <v>5</v>
-      </c>
+      <c r="H51" s="46" t="n"/>
       <c r="I51" s="21" t="n">
         <v>4</v>
       </c>
       <c r="J51" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K51" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K51" s="46" t="n"/>
       <c r="L51" s="22" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="M51" s="21" t="inlineStr">
         <is>
@@ -10691,20 +10595,16 @@
       <c r="G52" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H52" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H52" s="46" t="n"/>
       <c r="I52" s="21" t="n">
         <v>4</v>
       </c>
       <c r="J52" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K52" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K52" s="46" t="n"/>
       <c r="L52" s="25" t="n">
-        <v>3.8</v>
+        <v>3.67</v>
       </c>
       <c r="M52" s="23" t="inlineStr">
         <is>
@@ -10746,20 +10646,16 @@
       <c r="G53" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H53" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="H53" s="46" t="n"/>
       <c r="I53" s="21" t="n">
         <v>3</v>
       </c>
       <c r="J53" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="K53" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K53" s="46" t="n"/>
       <c r="L53" s="25" t="n">
-        <v>3</v>
+        <v>2.67</v>
       </c>
       <c r="M53" s="21" t="inlineStr">
         <is>
@@ -10801,20 +10697,16 @@
       <c r="G54" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H54" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H54" s="46" t="n"/>
       <c r="I54" s="21" t="n">
         <v>4</v>
       </c>
       <c r="J54" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K54" s="21" t="n">
-        <v>5</v>
-      </c>
+      <c r="K54" s="46" t="n"/>
       <c r="L54" s="22" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="M54" s="23" t="inlineStr">
         <is>
@@ -10856,18 +10748,14 @@
       <c r="G55" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H55" s="21" t="n">
-        <v>2</v>
-      </c>
+      <c r="H55" s="46" t="n"/>
       <c r="I55" s="21" t="n">
         <v>3</v>
       </c>
       <c r="J55" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="K55" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K55" s="46" t="n"/>
       <c r="L55" s="25" t="n">
         <v>3</v>
       </c>
@@ -10911,20 +10799,16 @@
       <c r="G56" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H56" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="H56" s="46" t="n"/>
       <c r="I56" s="21" t="n">
         <v>4</v>
       </c>
       <c r="J56" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K56" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K56" s="46" t="n"/>
       <c r="L56" s="25" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="M56" s="23" t="inlineStr">
         <is>
@@ -10966,18 +10850,14 @@
       <c r="G57" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H57" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H57" s="46" t="n"/>
       <c r="I57" s="21" t="n">
         <v>4</v>
       </c>
       <c r="J57" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K57" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K57" s="46" t="n"/>
       <c r="L57" s="22" t="n">
         <v>4</v>
       </c>
@@ -11021,18 +10901,14 @@
       <c r="G58" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H58" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="H58" s="46" t="n"/>
       <c r="I58" s="21" t="n">
         <v>3</v>
       </c>
       <c r="J58" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="K58" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="K58" s="46" t="n"/>
       <c r="L58" s="25" t="n">
         <v>3</v>
       </c>
@@ -11076,20 +10952,16 @@
       <c r="G59" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H59" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H59" s="46" t="n"/>
       <c r="I59" s="21" t="n">
         <v>4</v>
       </c>
       <c r="J59" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="K59" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K59" s="46" t="n"/>
       <c r="L59" s="22" t="n">
-        <v>4.2</v>
+        <v>4.33</v>
       </c>
       <c r="M59" s="21" t="inlineStr">
         <is>
@@ -11131,18 +11003,12 @@
       <c r="G60" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H60" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="I60" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H60" s="46" t="n"/>
+      <c r="I60" s="46" t="n"/>
       <c r="J60" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K60" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K60" s="46" t="n"/>
       <c r="L60" s="22" t="n">
         <v>4</v>
       </c>
@@ -11186,20 +11052,14 @@
       <c r="G61" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H61" s="21" t="n">
-        <v>5</v>
-      </c>
-      <c r="I61" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H61" s="46" t="n"/>
+      <c r="I61" s="46" t="n"/>
       <c r="J61" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K61" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K61" s="46" t="n"/>
       <c r="L61" s="22" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="M61" s="21" t="inlineStr">
         <is>
@@ -11241,20 +11101,14 @@
       <c r="G62" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H62" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="I62" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H62" s="46" t="n"/>
+      <c r="I62" s="46" t="n"/>
       <c r="J62" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K62" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K62" s="46" t="n"/>
       <c r="L62" s="25" t="n">
-        <v>3.8</v>
+        <v>3.5</v>
       </c>
       <c r="M62" s="23" t="inlineStr">
         <is>
@@ -11296,20 +11150,14 @@
       <c r="G63" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H63" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="I63" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H63" s="46" t="n"/>
+      <c r="I63" s="46" t="n"/>
       <c r="J63" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="K63" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K63" s="46" t="n"/>
       <c r="L63" s="22" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="M63" s="21" t="inlineStr">
         <is>
@@ -11351,20 +11199,14 @@
       <c r="G64" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H64" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="I64" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H64" s="46" t="n"/>
+      <c r="I64" s="46" t="n"/>
       <c r="J64" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K64" s="21" t="n">
-        <v>5</v>
-      </c>
+      <c r="K64" s="46" t="n"/>
       <c r="L64" s="22" t="n">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="M64" s="23" t="inlineStr">
         <is>
@@ -11406,20 +11248,14 @@
       <c r="G65" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H65" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="I65" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H65" s="46" t="n"/>
+      <c r="I65" s="46" t="n"/>
       <c r="J65" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K65" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K65" s="46" t="n"/>
       <c r="L65" s="25" t="n">
-        <v>3.8</v>
+        <v>4</v>
       </c>
       <c r="M65" s="21" t="inlineStr">
         <is>
@@ -11461,18 +11297,12 @@
       <c r="G66" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H66" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="I66" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H66" s="46" t="n"/>
+      <c r="I66" s="46" t="n"/>
       <c r="J66" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K66" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K66" s="46" t="n"/>
       <c r="L66" s="22" t="n">
         <v>4</v>
       </c>
@@ -11516,20 +11346,14 @@
       <c r="G67" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="H67" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="I67" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="H67" s="46" t="n"/>
+      <c r="I67" s="46" t="n"/>
       <c r="J67" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K67" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K67" s="46" t="n"/>
       <c r="L67" s="22" t="n">
-        <v>4.2</v>
+        <v>4.5</v>
       </c>
       <c r="M67" s="21" t="inlineStr">
         <is>
@@ -11571,20 +11395,14 @@
       <c r="G68" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="H68" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="I68" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="H68" s="46" t="n"/>
+      <c r="I68" s="46" t="n"/>
       <c r="J68" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="K68" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K68" s="46" t="n"/>
       <c r="L68" s="25" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="M68" s="23" t="inlineStr">
         <is>
@@ -11626,20 +11444,14 @@
       <c r="G69" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H69" s="21" t="n">
-        <v>5</v>
-      </c>
-      <c r="I69" s="21" t="n">
-        <v>5</v>
-      </c>
+      <c r="H69" s="46" t="n"/>
+      <c r="I69" s="46" t="n"/>
       <c r="J69" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K69" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="K69" s="46" t="n"/>
       <c r="L69" s="22" t="n">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="M69" s="21" t="inlineStr">
         <is>
@@ -11681,20 +11493,14 @@
       <c r="G70" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="H70" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="I70" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="H70" s="46" t="n"/>
+      <c r="I70" s="46" t="n"/>
       <c r="J70" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="K70" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="K70" s="46" t="n"/>
       <c r="L70" s="25" t="n">
-        <v>3.4</v>
+        <v>4</v>
       </c>
       <c r="M70" s="23" t="inlineStr">
         <is>
@@ -11739,17 +11545,13 @@
       <c r="H71" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="I71" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="J71" s="21" t="n">
-        <v>2</v>
-      </c>
+      <c r="I71" s="46" t="n"/>
+      <c r="J71" s="46" t="n"/>
       <c r="K71" s="21" t="n">
         <v>3</v>
       </c>
       <c r="L71" s="27" t="n">
-        <v>2.6</v>
+        <v>2.67</v>
       </c>
       <c r="M71" s="21" t="inlineStr">
         <is>
@@ -11794,12 +11596,8 @@
       <c r="H72" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I72" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J72" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I72" s="46" t="n"/>
+      <c r="J72" s="46" t="n"/>
       <c r="K72" s="21" t="n">
         <v>4</v>
       </c>
@@ -11849,17 +11647,13 @@
       <c r="H73" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="I73" s="21" t="n">
-        <v>2</v>
-      </c>
-      <c r="J73" s="21" t="n">
-        <v>1</v>
-      </c>
+      <c r="I73" s="46" t="n"/>
+      <c r="J73" s="46" t="n"/>
       <c r="K73" s="21" t="n">
         <v>1</v>
       </c>
       <c r="L73" s="29" t="n">
-        <v>1.4</v>
+        <v>1.33</v>
       </c>
       <c r="M73" s="21" t="inlineStr">
         <is>
@@ -11904,17 +11698,13 @@
       <c r="H74" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I74" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J74" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I74" s="46" t="n"/>
+      <c r="J74" s="46" t="n"/>
       <c r="K74" s="21" t="n">
         <v>4</v>
       </c>
       <c r="L74" s="25" t="n">
-        <v>3.8</v>
+        <v>3.67</v>
       </c>
       <c r="M74" s="23" t="inlineStr">
         <is>
@@ -11959,17 +11749,13 @@
       <c r="H75" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I75" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J75" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I75" s="46" t="n"/>
+      <c r="J75" s="46" t="n"/>
       <c r="K75" s="21" t="n">
         <v>5</v>
       </c>
       <c r="L75" s="22" t="n">
-        <v>4.2</v>
+        <v>4.33</v>
       </c>
       <c r="M75" s="21" t="inlineStr">
         <is>
@@ -12014,17 +11800,13 @@
       <c r="H76" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="I76" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J76" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I76" s="46" t="n"/>
+      <c r="J76" s="46" t="n"/>
       <c r="K76" s="21" t="n">
         <v>4</v>
       </c>
       <c r="L76" s="25" t="n">
-        <v>3.8</v>
+        <v>3.67</v>
       </c>
       <c r="M76" s="23" t="inlineStr">
         <is>
@@ -12069,17 +11851,13 @@
       <c r="H77" s="21" t="n">
         <v>2</v>
       </c>
-      <c r="I77" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="J77" s="21" t="n">
-        <v>1</v>
-      </c>
+      <c r="I77" s="46" t="n"/>
+      <c r="J77" s="46" t="n"/>
       <c r="K77" s="21" t="n">
         <v>2</v>
       </c>
       <c r="L77" s="29" t="n">
-        <v>1.4</v>
+        <v>1.67</v>
       </c>
       <c r="M77" s="21" t="inlineStr">
         <is>
@@ -12124,12 +11902,8 @@
       <c r="H78" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I78" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J78" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I78" s="46" t="n"/>
+      <c r="J78" s="46" t="n"/>
       <c r="K78" s="21" t="n">
         <v>4</v>
       </c>
@@ -12179,17 +11953,13 @@
       <c r="H79" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I79" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J79" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I79" s="46" t="n"/>
+      <c r="J79" s="46" t="n"/>
       <c r="K79" s="21" t="n">
         <v>4</v>
       </c>
       <c r="L79" s="25" t="n">
-        <v>3.8</v>
+        <v>3.67</v>
       </c>
       <c r="M79" s="21" t="inlineStr">
         <is>
@@ -12234,12 +12004,8 @@
       <c r="H80" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="I80" s="21" t="n">
-        <v>3</v>
-      </c>
-      <c r="J80" s="21" t="n">
-        <v>3</v>
-      </c>
+      <c r="I80" s="46" t="n"/>
+      <c r="J80" s="46" t="n"/>
       <c r="K80" s="21" t="n">
         <v>3</v>
       </c>
@@ -12289,17 +12055,13 @@
       <c r="H81" s="21" t="n">
         <v>4</v>
       </c>
-      <c r="I81" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J81" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I81" s="46" t="n"/>
+      <c r="J81" s="46" t="n"/>
       <c r="K81" s="21" t="n">
         <v>5</v>
       </c>
       <c r="L81" s="22" t="n">
-        <v>4.2</v>
+        <v>4.33</v>
       </c>
       <c r="M81" s="21" t="inlineStr">
         <is>
@@ -12344,17 +12106,13 @@
       <c r="H82" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="I82" s="21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J82" s="21" t="n">
-        <v>4</v>
-      </c>
+      <c r="I82" s="46" t="n"/>
+      <c r="J82" s="46" t="n"/>
       <c r="K82" s="21" t="n">
         <v>3</v>
       </c>
       <c r="L82" s="25" t="n">
-        <v>3.4</v>
+        <v>3</v>
       </c>
       <c r="M82" s="23" t="inlineStr">
         <is>

</xml_diff>